<commit_message>
avance 19-02-2025; se corrigen los errores de las rutas que acceden a los archivos xlsx
</commit_message>
<xml_diff>
--- a/Backend/output/informe_final.xlsx
+++ b/Backend/output/informe_final.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A589DDF-A1B3-4D04-B0F8-7571B51F8D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7D0C453-1C40-40B5-A102-EF7F24D3B70F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="733" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -823,7 +823,7 @@
     <t xml:space="preserve">RESULTADO EX ANTE </t>
   </si>
   <si>
-    <t>DICIEMBRE - 2024</t>
+    <t>ENERO - 2025</t>
   </si>
   <si>
     <t>Gab Subse</t>
@@ -1312,10 +1312,10 @@
     <t>En octubre se envió mediante mail del Jefe del Gabinete del Ministro, el resultado del monitoreo del segundo año de gestión.</t>
   </si>
   <si>
-    <t>Acum diciembre - 2024</t>
-  </si>
-  <si>
-    <t>Hitos ADP ocurridos al 24 de diciembre</t>
+    <t>Acum ENERO - 2025</t>
+  </si>
+  <si>
+    <t>Hitos ADP ocurridos al 19 de ENERO</t>
   </si>
   <si>
     <t>Política de Gestión de Riesgos</t>
@@ -12943,7 +12943,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{34998BFF-D8D2-4A8F-8593-A33373321E10}" type="CELLRANGE">
+                    <a:fld id="{EEC3284A-1D12-4541-B4BD-BC5C0CAAC136}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -12977,7 +12977,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{86CBE627-3C0F-4978-B0DC-4CFA59A5D826}" type="CELLRANGE">
+                    <a:fld id="{3901D9A8-1478-4896-969F-4536D65BC343}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13011,7 +13011,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E2CBA465-4450-4A78-8F16-A8FE2FD1AFED}" type="CELLRANGE">
+                    <a:fld id="{89ABB867-2256-409B-93C2-31E8A17EE74E}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13045,7 +13045,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2B249169-5BD0-4F1B-9198-701BA88C2814}" type="CELLRANGE">
+                    <a:fld id="{D8C0F4C1-2931-4292-91DE-3F3B8AC089FD}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13079,7 +13079,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A09EECD4-3F58-4FD5-87A0-EC873ED0D5A8}" type="CELLRANGE">
+                    <a:fld id="{6A19137B-2D14-4005-A000-15DCB4EFC1C2}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13113,7 +13113,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BF31348A-2324-42F9-A2F5-A5A3192E1D50}" type="CELLRANGE">
+                    <a:fld id="{277E8A87-E022-4A06-9D64-3F5FBEEEC105}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13147,7 +13147,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EFE3E381-F170-4180-AA96-5A4F340894B7}" type="CELLRANGE">
+                    <a:fld id="{CC6CF608-F57F-4350-99EA-68DF58399C14}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13181,7 +13181,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DB9DF5BE-AE12-4AB0-868D-263C01483CD3}" type="CELLRANGE">
+                    <a:fld id="{6918DFEB-DF5D-412E-BE16-08E4231F8D56}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13215,7 +13215,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2C1DB71A-F76F-4960-AF58-51177E7FD95F}" type="CELLRANGE">
+                    <a:fld id="{B1D51C0B-F48B-4E2D-821E-FE94A8716AD4}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13249,7 +13249,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0FF58543-30B4-4B02-83DA-D9E978168D83}" type="CELLRANGE">
+                    <a:fld id="{8845C194-D043-44F6-A8D1-0DF940D3D360}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13283,7 +13283,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6EA55170-8142-482D-90DE-A1EE59C7E261}" type="CELLRANGE">
+                    <a:fld id="{C73A5DF3-B07C-4689-B046-EBAAB7944AFF}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13317,7 +13317,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DA8A8286-A200-4A63-947D-9969200E2BF2}" type="CELLRANGE">
+                    <a:fld id="{2855ABBC-6F3F-4CD1-BB59-F28358BC5072}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13694,7 +13694,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{31A588B1-9C89-493D-AF7D-F2A84DDEC711}" type="CELLRANGE">
+                    <a:fld id="{C0487E3F-585E-455E-B519-817CFBD4B253}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -14418,7 +14418,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{31FBFC7A-C227-44A6-B6E5-9F1BF52B6A97}" type="CELLRANGE">
+                    <a:fld id="{DA9C1530-8952-40FB-B247-F96B093B8736}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr>
                         <a:defRPr sz="1400">
@@ -14499,7 +14499,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{74D90ABB-66FC-41FE-9269-A82190059F92}" type="CELLRANGE">
+                    <a:fld id="{C03A957D-69DF-4E86-96F4-5067CAF52B61}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -27083,7 +27083,7 @@
         <v>193</v>
       </c>
       <c r="G11" s="458">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="H11" s="458"/>
       <c r="I11" s="125"/>
@@ -33327,7 +33327,7 @@
       <c r="A8" s="44"/>
       <c r="C8" s="473" t="str">
         <f>_xlfn.CONCAT("PERIODO ", N5)</f>
-        <v>PERIODO DICIEMBRE - 2024</v>
+        <v>PERIODO ENERO - 2025</v>
       </c>
       <c r="D8" s="474"/>
       <c r="E8" s="475"/>

</xml_diff>

<commit_message>
avance 24-03-25; se da corrección al error de bordes y formatos del anexo indicadores
</commit_message>
<xml_diff>
--- a/Backend/output/informe_final.xlsx
+++ b/Backend/output/informe_final.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8BDD170-A9EF-41E2-8339-2798E0624F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D85C889-B46F-47A7-9122-354427E1C8F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="733" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1283,7 +1283,7 @@
     <t>Acum FEBRERO - 2025</t>
   </si>
   <si>
-    <t>Hitos ADP ocurridos al 21 de FEBRERO</t>
+    <t>Hitos ADP ocurridos al 24 de FEBRERO</t>
   </si>
   <si>
     <t>Política de Gestión de Riesgos</t>
@@ -12978,7 +12978,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3175E1D9-2D5D-4C98-A330-AE0EF765B1FB}" type="CELLRANGE">
+                    <a:fld id="{79B59CAE-E957-4DB4-A03E-A3EE21D9F64F}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13012,7 +13012,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A15D19F6-B3A8-42D4-9634-38BB377AB6AA}" type="CELLRANGE">
+                    <a:fld id="{E8770FB4-C04F-416A-96BB-97FEC533CD48}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13046,7 +13046,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{29E652C9-5A2E-4A1C-A4F3-AAEAE0F28D73}" type="CELLRANGE">
+                    <a:fld id="{D17A1A71-7EA6-4C96-80A3-F5A7805C2BEF}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13080,7 +13080,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{25E5A8A0-1677-430D-9D51-A0D4F3E53949}" type="CELLRANGE">
+                    <a:fld id="{3F104E5E-D0D6-44EE-9E91-54EFC0A0BE7B}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13114,7 +13114,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AB18087C-B0B4-4FDA-B8D3-97E1A4C7F925}" type="CELLRANGE">
+                    <a:fld id="{C889C164-6AEA-4671-8BBC-6DB2F3607B95}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13148,7 +13148,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5A8A8B55-3E58-4904-B1FF-D5B4C278A9CD}" type="CELLRANGE">
+                    <a:fld id="{ADE2AA2F-A697-4162-856B-43AFA0CBAB2E}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13182,7 +13182,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{74C8F4BF-18EC-4703-A454-CD4C9BCB682C}" type="CELLRANGE">
+                    <a:fld id="{AEE85172-3D79-4A05-A699-0FAB2EE80C9C}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13216,7 +13216,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1677952B-0432-4CAD-909C-7909772240D4}" type="CELLRANGE">
+                    <a:fld id="{DC14568C-9879-4365-B22E-164EB210BF5B}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13250,7 +13250,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5B3C83E3-6461-45E8-B140-8A63C65E3081}" type="CELLRANGE">
+                    <a:fld id="{9422167C-3C91-4C25-805D-0245CE8E921F}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13284,7 +13284,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5B33D0CF-087A-405F-A2C3-C5F8DA68EED1}" type="CELLRANGE">
+                    <a:fld id="{84FC4139-BE11-4712-BFE8-04AB590DD951}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13318,7 +13318,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7A9CB30D-2948-4BA6-8522-35849B103305}" type="CELLRANGE">
+                    <a:fld id="{03A51483-CE80-4FF0-945E-DEA92855A65E}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13352,7 +13352,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3962EFBA-CD79-4E74-B811-50A0C808E94E}" type="CELLRANGE">
+                    <a:fld id="{CAFC47C8-942C-494C-8F8A-0DF2225280BD}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13729,7 +13729,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FBA4F8E7-DEBE-4EA4-8C13-5B51D231F7D4}" type="CELLRANGE">
+                    <a:fld id="{6D2371AD-21AA-4185-BF32-E016B0499682}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -14453,7 +14453,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{EC229AEE-9755-41C2-8D28-EA5B2D1F5154}" type="CELLRANGE">
+                    <a:fld id="{1EA9646C-584E-4176-BC78-1B3D073BBEED}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr>
                         <a:defRPr sz="1400">
@@ -14534,7 +14534,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2C8E3F93-9497-42E9-8E23-FADEAA05BDD0}" type="CELLRANGE">
+                    <a:fld id="{F1714C22-BDEE-449A-A289-3803D3E1DFFD}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>

</xml_diff>

<commit_message>
avance 26-03-25; se corrigen errores de graficos
</commit_message>
<xml_diff>
--- a/Backend/output/informe_final.xlsx
+++ b/Backend/output/informe_final.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D85C889-B46F-47A7-9122-354427E1C8F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BB42F77-4B96-4773-A06C-0B978915D389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="733" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="15375" windowHeight="7785" tabRatio="733" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="52" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="426">
   <si>
     <t>SUBSECRETARÍA DE EDUCACIÓN</t>
   </si>
@@ -851,45 +851,12 @@
     <t>I20_014-Gabinete Ministerio</t>
   </si>
   <si>
-    <t>PTR25_040-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_041-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_042-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_043-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_044-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_053-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_054-Gabinete Ministerio</t>
-  </si>
-  <si>
-    <t>PTR25_055-Gabinete Ministerio</t>
-  </si>
-  <si>
     <t>I19_026-Gabinete Subsecretaría</t>
   </si>
   <si>
     <t>I23_015-Gabinete Subsecretaría</t>
   </si>
   <si>
-    <t>PTR25_045-Gabinete Subsecretaría</t>
-  </si>
-  <si>
-    <t>PTR25_046-Gabinete Subsecretaría</t>
-  </si>
-  <si>
-    <t>PTR25_047-Gabinete Subsecretaría</t>
-  </si>
-  <si>
     <t>I21_001-Gabinete Subsecretaría</t>
   </si>
   <si>
@@ -905,24 +872,6 @@
     <t>I23_018-CPEIP</t>
   </si>
   <si>
-    <t>PTR25_001-CPEIP</t>
-  </si>
-  <si>
-    <t>PTR25_002-CPEIP</t>
-  </si>
-  <si>
-    <t>PTR25_003-CPEIP</t>
-  </si>
-  <si>
-    <t>PTR25_004-CPEIP</t>
-  </si>
-  <si>
-    <t>PTR25_005-CPEIP</t>
-  </si>
-  <si>
-    <t>PTR25_006-CPEIP</t>
-  </si>
-  <si>
     <t>I25_003-CPEIP</t>
   </si>
   <si>
@@ -932,25 +881,97 @@
     <t>I25_011-DEG</t>
   </si>
   <si>
-    <t>PTR25_015-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_016-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_017-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_018-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_019-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_020-DEG</t>
-  </si>
-  <si>
-    <t>PTR25_021-DEG</t>
+    <t>I17_001-DEG</t>
+  </si>
+  <si>
+    <t>I23_004-DEG</t>
+  </si>
+  <si>
+    <t>I24_009-DEG</t>
+  </si>
+  <si>
+    <t>I16_043-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I20_011-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I20_012-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I25_012-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I21_002-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I16_054-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I19_012-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I25_005-División de Planificación y Presupuesto</t>
+  </si>
+  <si>
+    <t>I21_007-DAG</t>
+  </si>
+  <si>
+    <t>I25_004-DAG</t>
+  </si>
+  <si>
+    <t>I23_019-DAG</t>
+  </si>
+  <si>
+    <t>I25_013-DAG</t>
+  </si>
+  <si>
+    <t>I20_006-DAG</t>
+  </si>
+  <si>
+    <t>I20_005-DAG</t>
+  </si>
+  <si>
+    <t>I19_020-UCE</t>
+  </si>
+  <si>
+    <t>I21_011-UCE</t>
+  </si>
+  <si>
+    <t>I21_012-UCE</t>
+  </si>
+  <si>
+    <t>I22_006-UCE</t>
+  </si>
+  <si>
+    <t>I19_019-UCE</t>
+  </si>
+  <si>
+    <t>I16_062-UCE</t>
+  </si>
+  <si>
+    <t>I25_010-UCE</t>
+  </si>
+  <si>
+    <t>I16_052-División Jurídica</t>
+  </si>
+  <si>
+    <t>I24_004-División Jurídica</t>
+  </si>
+  <si>
+    <t>I23_007-División Jurídica</t>
+  </si>
+  <si>
+    <t>I22_008-División Jurídica</t>
+  </si>
+  <si>
+    <t>I24_011-División Jurídica</t>
+  </si>
+  <si>
+    <t>I24_003-División Jurídica</t>
+  </si>
+  <si>
+    <t>I16_053-División Jurídica</t>
   </si>
   <si>
     <t>Sin dato</t>
@@ -1283,7 +1304,7 @@
     <t>Acum FEBRERO - 2025</t>
   </si>
   <si>
-    <t>Hitos ADP ocurridos al 24 de FEBRERO</t>
+    <t>Hitos ADP ocurridos al 26 de FEBRERO</t>
   </si>
   <si>
     <t>Política de Gestión de Riesgos</t>
@@ -12978,7 +12999,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{79B59CAE-E957-4DB4-A03E-A3EE21D9F64F}" type="CELLRANGE">
+                    <a:fld id="{5B07F8DF-8178-4A03-A2B6-C18807156040}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13012,7 +13033,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E8770FB4-C04F-416A-96BB-97FEC533CD48}" type="CELLRANGE">
+                    <a:fld id="{67C5E621-8048-4CC9-B507-8CF5753626C5}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13046,7 +13067,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D17A1A71-7EA6-4C96-80A3-F5A7805C2BEF}" type="CELLRANGE">
+                    <a:fld id="{AB6BEC96-EE4D-48CA-88A5-6EF718249E2D}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13080,7 +13101,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3F104E5E-D0D6-44EE-9E91-54EFC0A0BE7B}" type="CELLRANGE">
+                    <a:fld id="{9E4C2A99-CF5A-41E8-97A7-83E2C3F39317}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13114,7 +13135,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C889C164-6AEA-4671-8BBC-6DB2F3607B95}" type="CELLRANGE">
+                    <a:fld id="{5378AA3C-52DC-4ADE-9928-1EB2C6FC1D90}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13148,7 +13169,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ADE2AA2F-A697-4162-856B-43AFA0CBAB2E}" type="CELLRANGE">
+                    <a:fld id="{7F2B2987-2056-4900-B547-FCF4720D72CE}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13182,7 +13203,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AEE85172-3D79-4A05-A699-0FAB2EE80C9C}" type="CELLRANGE">
+                    <a:fld id="{F1DD95AE-F0D5-4125-AAE6-273816F56566}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13216,7 +13237,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DC14568C-9879-4365-B22E-164EB210BF5B}" type="CELLRANGE">
+                    <a:fld id="{F7FC12B3-95C8-410F-8401-C49B73A1CB61}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13250,7 +13271,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9422167C-3C91-4C25-805D-0245CE8E921F}" type="CELLRANGE">
+                    <a:fld id="{1A582626-5512-4C00-81D9-B3C20FAA95CB}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13284,7 +13305,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{84FC4139-BE11-4712-BFE8-04AB590DD951}" type="CELLRANGE">
+                    <a:fld id="{48838F0F-4E8E-449F-AA01-B17679F72977}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13318,7 +13339,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{03A51483-CE80-4FF0-945E-DEA92855A65E}" type="CELLRANGE">
+                    <a:fld id="{559B87D9-0052-41DE-A66D-638DB3F8626B}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13352,7 +13373,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CAFC47C8-942C-494C-8F8A-0DF2225280BD}" type="CELLRANGE">
+                    <a:fld id="{1598D04A-8C0F-488C-A87D-F7DC68393B39}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -13729,7 +13750,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6D2371AD-21AA-4185-BF32-E016B0499682}" type="CELLRANGE">
+                    <a:fld id="{3B5E661A-7FAA-4F8D-8BA9-AF3A173149C2}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -14453,7 +14474,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{1EA9646C-584E-4176-BC78-1B3D073BBEED}" type="CELLRANGE">
+                    <a:fld id="{9225CDDF-8E27-4A2E-BB9F-DAB4EC5C1D8D}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr>
                         <a:defRPr sz="1400">
@@ -14534,7 +14555,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F1714C22-BDEE-449A-A289-3803D3E1DFFD}" type="CELLRANGE">
+                    <a:fld id="{ED06BA52-1CFC-42CC-8BB9-F8F874D9BD1A}" type="CELLRANGE">
                       <a:rPr lang="es-CL"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -28195,10 +28216,10 @@
     <row r="8" spans="1:28" ht="21.75" customHeight="1" thickBot="1">
       <c r="A8" s="209"/>
       <c r="B8" s="221" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="D8" s="210">
         <v>2019</v>
@@ -28230,10 +28251,10 @@
     <row r="9" spans="1:28" ht="18" customHeight="1" thickBot="1">
       <c r="A9" s="214"/>
       <c r="B9" s="221" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="C9" s="216" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D9" s="160">
         <v>2024</v>
@@ -28265,10 +28286,10 @@
     <row r="10" spans="1:28" ht="21" customHeight="1">
       <c r="A10" s="97"/>
       <c r="B10" s="221" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="C10" s="216" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D10" s="160">
         <v>2024</v>
@@ -28302,10 +28323,10 @@
     <row r="11" spans="1:28" ht="19.5" customHeight="1">
       <c r="A11" s="95"/>
       <c r="B11" s="221" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C11" s="220" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D11" s="160">
         <v>2024</v>
@@ -28347,10 +28368,10 @@
     <row r="12" spans="1:28" ht="17.25" customHeight="1">
       <c r="A12" s="95"/>
       <c r="B12" s="222" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="C12" s="224" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D12" s="216">
         <v>2024</v>
@@ -28390,10 +28411,10 @@
     <row r="13" spans="1:28" ht="18.75" customHeight="1">
       <c r="A13" s="95"/>
       <c r="B13" s="221" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D13" s="160">
         <v>2024</v>
@@ -28425,10 +28446,10 @@
     <row r="14" spans="1:28" ht="18.75" customHeight="1">
       <c r="A14" s="95"/>
       <c r="B14" s="221" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="C14" s="216" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D14" s="160">
         <v>2024</v>
@@ -28475,10 +28496,10 @@
     <row r="15" spans="1:28" ht="19.5" customHeight="1" thickBot="1">
       <c r="A15" s="95"/>
       <c r="B15" s="223" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="C15" s="218" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D15" s="217">
         <v>2024</v>
@@ -28632,7 +28653,7 @@
       </c>
       <c r="F18" s="105"/>
       <c r="G18" s="623" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="H18" s="624"/>
       <c r="I18" s="601">
@@ -28678,12 +28699,12 @@
         <v>16</v>
       </c>
       <c r="D19" s="165" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E19" s="233"/>
       <c r="F19" s="105"/>
       <c r="G19" s="623" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="H19" s="624"/>
       <c r="I19" s="601">
@@ -28729,7 +28750,7 @@
         <v>13</v>
       </c>
       <c r="D20" s="165" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E20" s="233"/>
       <c r="F20" s="105"/>
@@ -28774,13 +28795,13 @@
     <row r="21" spans="1:27" ht="30" customHeight="1">
       <c r="A21" s="95"/>
       <c r="B21" s="185" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="C21" s="165">
         <v>35</v>
       </c>
       <c r="D21" s="165" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E21" s="233"/>
       <c r="F21" s="105"/>
@@ -28831,12 +28852,12 @@
         <v>21</v>
       </c>
       <c r="D22" s="165" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E22" s="233"/>
       <c r="F22" s="105"/>
       <c r="G22" s="623" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="H22" s="624"/>
       <c r="I22" s="601">
@@ -28876,13 +28897,13 @@
     <row r="23" spans="1:27" ht="30.75" customHeight="1" thickBot="1">
       <c r="A23" s="95"/>
       <c r="B23" s="186" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="C23" s="187">
         <v>2</v>
       </c>
       <c r="D23" s="187" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E23" s="234"/>
       <c r="F23" s="105"/>
@@ -29297,7 +29318,7 @@
       <c r="J33" s="550"/>
       <c r="K33" s="105"/>
       <c r="L33" s="583" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="M33" s="551"/>
       <c r="N33" s="551"/>
@@ -29342,7 +29363,7 @@
       <c r="J34" s="193"/>
       <c r="K34" s="105"/>
       <c r="L34" s="583" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="M34" s="551"/>
       <c r="N34" s="551"/>
@@ -29479,7 +29500,7 @@
       <c r="J37" s="574"/>
       <c r="K37" s="105"/>
       <c r="L37" s="583" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="M37" s="551"/>
       <c r="N37" s="552"/>
@@ -31855,7 +31876,7 @@
       </c>
       <c r="L6" s="679"/>
       <c r="M6" s="698" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="N6" s="679"/>
       <c r="O6" s="698" t="s">
@@ -31883,7 +31904,7 @@
       </c>
       <c r="L7" s="671"/>
       <c r="M7" s="670" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="N7" s="671"/>
       <c r="O7" s="670" t="s">
@@ -31908,7 +31929,7 @@
       </c>
       <c r="L8" s="671"/>
       <c r="M8" s="670" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="N8" s="671"/>
       <c r="O8" s="670" t="s">
@@ -31933,7 +31954,7 @@
       </c>
       <c r="L9" s="671"/>
       <c r="M9" s="670" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="N9" s="671"/>
       <c r="O9" s="670" t="s">
@@ -31958,7 +31979,7 @@
       </c>
       <c r="L10" s="671"/>
       <c r="M10" s="670" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="N10" s="671"/>
       <c r="O10" s="670" t="s">
@@ -31985,11 +32006,11 @@
       <c r="I11" s="96"/>
       <c r="J11" s="119"/>
       <c r="K11" s="674" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="L11" s="671"/>
       <c r="M11" s="670" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="N11" s="671"/>
       <c r="O11" s="670" t="s">
@@ -32018,15 +32039,15 @@
       <c r="I12" s="96"/>
       <c r="J12" s="119"/>
       <c r="K12" s="674" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="L12" s="671"/>
       <c r="M12" s="670" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="N12" s="671"/>
       <c r="O12" s="670" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="P12" s="677"/>
       <c r="Q12" s="96"/>
@@ -32051,11 +32072,11 @@
       <c r="I13" s="96"/>
       <c r="J13" s="95"/>
       <c r="K13" s="674" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="L13" s="671"/>
       <c r="M13" s="670" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="N13" s="671"/>
       <c r="O13" s="670" t="s">
@@ -32084,11 +32105,11 @@
       <c r="I14" s="96"/>
       <c r="J14" s="103"/>
       <c r="K14" s="674" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="L14" s="671"/>
       <c r="M14" s="670" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="N14" s="671"/>
       <c r="O14" s="670" t="s">
@@ -32121,7 +32142,7 @@
       </c>
       <c r="L15" s="671"/>
       <c r="M15" s="670" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="N15" s="671"/>
       <c r="O15" s="670" t="s">
@@ -32154,7 +32175,7 @@
       </c>
       <c r="L16" s="671"/>
       <c r="M16" s="670" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="N16" s="671"/>
       <c r="O16" s="670" t="s">
@@ -32185,11 +32206,11 @@
       </c>
       <c r="L17" s="671"/>
       <c r="M17" s="670" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="N17" s="671"/>
       <c r="O17" s="670" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="P17" s="677"/>
       <c r="Q17" s="96"/>
@@ -32217,11 +32238,11 @@
       </c>
       <c r="L18" s="673"/>
       <c r="M18" s="672" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="N18" s="673"/>
       <c r="O18" s="672" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="P18" s="676"/>
       <c r="Q18" s="96"/>
@@ -33016,7 +33037,7 @@
         <v>45646</v>
       </c>
       <c r="B3" s="320" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C3" s="191">
         <v>2</v>
@@ -33030,7 +33051,7 @@
         <v>45294</v>
       </c>
       <c r="B4" s="320" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="C4" s="191">
         <v>-1</v>
@@ -33044,7 +33065,7 @@
         <v>45317</v>
       </c>
       <c r="B5" s="320" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C5" s="191">
         <v>1.5</v>
@@ -33058,7 +33079,7 @@
         <v>45677</v>
       </c>
       <c r="B6" s="320" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="C6" s="191">
         <v>-1</v>
@@ -33072,7 +33093,7 @@
         <v>45748</v>
       </c>
       <c r="B7" s="320" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="C7" s="191">
         <v>1</v>
@@ -33086,7 +33107,7 @@
         <v>45796</v>
       </c>
       <c r="B8" s="320" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C8" s="191">
         <v>2</v>
@@ -33100,7 +33121,7 @@
         <v>45432</v>
       </c>
       <c r="B9" s="320" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C9" s="191">
         <v>1</v>
@@ -33114,7 +33135,7 @@
         <v>45435</v>
       </c>
       <c r="B10" s="320" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C10" s="191">
         <v>-1</v>
@@ -33128,7 +33149,7 @@
         <v>45442</v>
       </c>
       <c r="B11" s="320" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C11" s="191">
         <v>-1</v>
@@ -33142,7 +33163,7 @@
         <v>45449</v>
       </c>
       <c r="B12" s="320" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C12" s="191">
         <v>-1</v>
@@ -33156,7 +33177,7 @@
         <v>45456</v>
       </c>
       <c r="B13" s="320" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="C13" s="191">
         <v>-1</v>
@@ -33170,7 +33191,7 @@
         <v>45463</v>
       </c>
       <c r="B14" s="320" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="C14" s="191">
         <v>1</v>
@@ -37304,10 +37325,10 @@
       <c r="D6" s="5"/>
       <c r="E6" s="4"/>
       <c r="I6" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="18" customHeight="1">
@@ -37318,16 +37339,16 @@
       <c r="C7" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="5" t="str">
+      <c r="D7" s="5">
         <f>IF(J9="bajo",0,IF(J9="medio",0.5,IF(J9="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E7" s="4"/>
       <c r="I7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1">
@@ -37342,10 +37363,10 @@
       </c>
       <c r="E8" s="4"/>
       <c r="I8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1">
@@ -37360,10 +37381,10 @@
       </c>
       <c r="E9" s="4"/>
       <c r="I9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="18" customHeight="1">
@@ -37372,16 +37393,16 @@
       <c r="C10" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="5" t="str">
+      <c r="D10" s="5">
         <f>IF(J10="bajo",0,IF(J10="medio",0.5,IF(J10="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E10" s="4"/>
       <c r="I10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="18" customHeight="1">
@@ -37390,16 +37411,16 @@
       <c r="C11" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="5" t="str">
+      <c r="D11" s="5">
         <f>IF(J12="bajo",0,IF(J12="medio",0.5,IF(J12="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E11" s="4"/>
       <c r="I11" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1">
@@ -37408,16 +37429,16 @@
       <c r="C12" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="5" t="str">
+      <c r="D12" s="5">
         <f>IF(J13="bajo",0,IF(J13="medio",0.5,IF(J13="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4"/>
       <c r="I12" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="18" customHeight="1">
@@ -37426,16 +37447,16 @@
       <c r="C13" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="5" t="str">
+      <c r="D13" s="5">
         <f>IF(J11="bajo",0,IF(J11="medio",0.5,IF(J11="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E13" s="4"/>
       <c r="I13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="18" customHeight="1">
@@ -37445,7 +37466,7 @@
       <c r="D14" s="5"/>
       <c r="E14" s="4"/>
       <c r="I14" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>13</v>
@@ -37459,13 +37480,13 @@
       <c r="C15" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="5" t="str">
+      <c r="D15" s="5">
         <f>IF(J18="bajo",0,IF(J18="medio",0.5,IF(J18="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E15" s="4"/>
       <c r="I15" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>13</v>
@@ -37477,13 +37498,13 @@
       <c r="C16" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="5" t="str">
+      <c r="D16" s="5">
         <f>IF(J17="bajo",0,IF(J17="medio",0.5,IF(J17="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E16" s="4"/>
       <c r="I16" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>13</v>
@@ -37495,16 +37516,16 @@
       <c r="C17" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="5" t="str">
+      <c r="D17" s="5">
         <f>IF(J19="bajo",0,IF(J19="medio",0.5,IF(J19="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E17" s="4"/>
       <c r="I17" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="21">
@@ -37519,10 +37540,10 @@
       </c>
       <c r="E18" s="4"/>
       <c r="I18" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="18" customHeight="1">
@@ -37532,10 +37553,10 @@
       <c r="D19" s="5"/>
       <c r="E19" s="4"/>
       <c r="I19" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="18" customHeight="1">
@@ -37546,16 +37567,16 @@
       <c r="C20" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="5" t="str">
+      <c r="D20" s="5">
         <f>IF(J22="bajo",0,IF(J22="medio",0.5,IF(J22="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E20" s="4"/>
       <c r="I20" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="18" customHeight="1">
@@ -37564,16 +37585,16 @@
       <c r="C21" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="5" t="str">
+      <c r="D21" s="5">
         <f>IF(J24="bajo",0,IF(J24="medio",0.5,IF(J24="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E21" s="4"/>
       <c r="I21" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="18" customHeight="1">
@@ -37582,16 +37603,16 @@
       <c r="C22" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="5" t="str">
+      <c r="D22" s="5">
         <f>IF(J23="bajo",0,IF(J23="medio",0.5,IF(J23="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E22" s="4"/>
       <c r="I22" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="18" customHeight="1">
@@ -37600,16 +37621,16 @@
       <c r="C23" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="5" t="str">
+      <c r="D23" s="5">
         <f>IF(J21="bajo",0,IF(J21="medio",0.5,IF(J21="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E23" s="4"/>
       <c r="I23" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="18" customHeight="1">
@@ -37618,16 +37639,16 @@
       <c r="C24" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="5" t="str">
+      <c r="D24" s="5">
         <f>IF(J20="bajo",0,IF(J20="medio",0.5,IF(J20="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E24" s="4"/>
       <c r="I24" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1">
@@ -37637,7 +37658,7 @@
       <c r="D25" s="5"/>
       <c r="E25" s="4"/>
       <c r="I25" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>13</v>
@@ -37651,13 +37672,13 @@
       <c r="C26" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="5" t="str">
+      <c r="D26" s="5">
         <f>IF(J27="bajo",0,IF(J27="medio",0.5,IF(J27="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E26" s="4"/>
       <c r="I26" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>13</v>
@@ -37675,10 +37696,10 @@
       </c>
       <c r="E27" s="4"/>
       <c r="I27" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="18" customHeight="1">
@@ -37693,10 +37714,10 @@
       </c>
       <c r="E28" s="4"/>
       <c r="I28" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1">
@@ -37711,10 +37732,10 @@
       </c>
       <c r="E29" s="4"/>
       <c r="I29" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="18" customHeight="1">
@@ -37729,7 +37750,7 @@
       </c>
       <c r="E30" s="4"/>
       <c r="I30" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="J30" s="6" t="s">
         <v>13</v>
@@ -37747,7 +37768,7 @@
       </c>
       <c r="E31" s="4"/>
       <c r="I31" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>13</v>
@@ -37759,13 +37780,13 @@
       <c r="C32" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="5" t="str">
+      <c r="D32" s="5">
         <f>IF(J28="bajo",0,IF(J28="medio",0.5,IF(J28="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E32" s="4"/>
       <c r="I32" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>13</v>
@@ -37783,7 +37804,7 @@
       </c>
       <c r="E33" s="4"/>
       <c r="I33" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="J33" s="6" t="s">
         <v>13</v>
@@ -37796,7 +37817,7 @@
       <c r="D34" s="5"/>
       <c r="E34" s="4"/>
       <c r="I34" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="J34" s="6" t="s">
         <v>13</v>
@@ -37816,10 +37837,10 @@
       </c>
       <c r="E35" s="4"/>
       <c r="I35" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1">
@@ -37834,10 +37855,10 @@
       </c>
       <c r="E36" s="4"/>
       <c r="I36" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="18" customHeight="1">
@@ -37846,16 +37867,16 @@
       <c r="C37" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="D37" s="5" t="str">
+      <c r="D37" s="5">
         <f>IF(J36="bajo",0,IF(J36="medio",0.5,IF(J36="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E37" s="4"/>
       <c r="I37" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="18" customHeight="1">
@@ -37864,16 +37885,16 @@
       <c r="C38" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="D38" s="5" t="str">
+      <c r="D38" s="5">
         <f>IF(J37="bajo",0,IF(J37="medio",0.5,IF(J37="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E38" s="4"/>
       <c r="I38" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="18" customHeight="1">
@@ -37882,16 +37903,16 @@
       <c r="C39" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="D39" s="5" t="str">
+      <c r="D39" s="5">
         <f>IF(J35="bajo",0,IF(J35="medio",0.5,IF(J35="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E39" s="4"/>
       <c r="I39" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="18" customHeight="1">
@@ -37901,10 +37922,10 @@
       <c r="D40" s="5"/>
       <c r="E40" s="4"/>
       <c r="I40" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="18" customHeight="1">
@@ -37915,13 +37936,13 @@
       <c r="C41" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="D41" s="5" t="str">
+      <c r="D41" s="5">
         <f>IF(J38="bajo",0,IF(J38="medio",0.5,IF(J38="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E41" s="4"/>
       <c r="I41" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>13</v>
@@ -37933,13 +37954,13 @@
       <c r="C42" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="D42" s="5" t="str">
+      <c r="D42" s="5">
         <f>IF(J39="bajo",0,IF(J39="medio",0.5,IF(J39="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E42" s="4"/>
       <c r="I42" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="J42" s="6" t="s">
         <v>13</v>
@@ -37951,13 +37972,13 @@
       <c r="C43" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="D43" s="5" t="str">
+      <c r="D43" s="5">
         <f>IF(J40="bajo",0,IF(J40="medio",0.5,IF(J40="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E43" s="4"/>
       <c r="I43" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>13</v>
@@ -37975,10 +37996,10 @@
       </c>
       <c r="E44" s="4"/>
       <c r="I44" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="18" customHeight="1">
@@ -37993,10 +38014,10 @@
       </c>
       <c r="E45" s="4"/>
       <c r="I45" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="20.25" customHeight="1">
@@ -38011,10 +38032,10 @@
       </c>
       <c r="E46" s="4"/>
       <c r="I46" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="18" customHeight="1">
@@ -38024,10 +38045,10 @@
       <c r="D47" s="5"/>
       <c r="E47" s="4"/>
       <c r="I47" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="18" customHeight="1">
@@ -38038,16 +38059,16 @@
       <c r="C48" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="D48" s="5" t="str">
+      <c r="D48" s="5">
         <f>IF(J49="bajo",0,IF(J49="medio",0.5,IF(J49="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E48" s="4"/>
       <c r="I48" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="18" customHeight="1">
@@ -38056,16 +38077,16 @@
       <c r="C49" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="5" t="str">
+      <c r="D49" s="5">
         <f>IF(J44="bajo",0,IF(J44="medio",0.5,IF(J44="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E49" s="4"/>
       <c r="I49" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="18" customHeight="1">
@@ -38074,17 +38095,11 @@
       <c r="C50" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="D50" s="5" t="str">
+      <c r="D50" s="5">
         <f>IF(J46="bajo",0,IF(J46="medio",0.5,IF(J46="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E50" s="4"/>
-      <c r="I50" t="s">
-        <v>263</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>264</v>
-      </c>
     </row>
     <row r="51" spans="1:10" ht="18" customHeight="1">
       <c r="A51" s="15"/>
@@ -38092,9 +38107,9 @@
       <c r="C51" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="D51" s="5" t="str">
+      <c r="D51" s="5">
         <f>IF(J47="bajo",0,IF(J47="medio",0.5,IF(J47="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E51" s="4"/>
     </row>
@@ -38104,9 +38119,9 @@
       <c r="C52" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="D52" s="5" t="str">
+      <c r="D52" s="5">
         <f>IF(J48="bajo",0,IF(J48="medio",0.5,IF(J48="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E52" s="4"/>
     </row>
@@ -38116,9 +38131,9 @@
       <c r="C53" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="D53" s="5" t="str">
+      <c r="D53" s="5">
         <f>IF(J45="bajo",0,IF(J45="medio",0.5,IF(J45="alto",1,"falta riesgo")))</f>
-        <v>falta riesgo</v>
+        <v>0</v>
       </c>
       <c r="E53" s="4"/>
     </row>
@@ -38206,10 +38221,10 @@
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>23</v>
@@ -38220,10 +38235,10 @@
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>24</v>
@@ -38234,10 +38249,10 @@
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
@@ -38248,10 +38263,10 @@
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>26</v>
@@ -38262,10 +38277,10 @@
     </row>
     <row r="8" spans="2:5">
       <c r="B8" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>27</v>
@@ -38276,10 +38291,10 @@
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>28</v>
@@ -38290,10 +38305,10 @@
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>29</v>
@@ -38304,10 +38319,10 @@
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>30</v>
@@ -38318,10 +38333,10 @@
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>226</v>
@@ -38332,10 +38347,10 @@
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>32</v>
@@ -38346,10 +38361,10 @@
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>33</v>
@@ -38360,10 +38375,10 @@
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>34</v>
@@ -38374,10 +38389,10 @@
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>35</v>
@@ -38388,10 +38403,10 @@
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>36</v>
@@ -38402,10 +38417,10 @@
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>37</v>
@@ -38416,10 +38431,10 @@
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>38</v>
@@ -38430,10 +38445,10 @@
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C20" s="90" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D20" s="90" t="s">
         <v>23</v>
@@ -38444,10 +38459,10 @@
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C21" s="90" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="D21" s="90" t="s">
         <v>24</v>
@@ -38458,10 +38473,10 @@
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C22" s="90" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D22" s="90" t="s">
         <v>25</v>
@@ -38472,10 +38487,10 @@
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C23" s="90" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D23" s="90" t="s">
         <v>26</v>
@@ -38486,10 +38501,10 @@
     </row>
     <row r="24" spans="2:5">
       <c r="B24" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C24" s="90" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D24" s="90" t="s">
         <v>27</v>
@@ -38500,10 +38515,10 @@
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C25" s="90" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D25" s="90" t="s">
         <v>28</v>
@@ -38514,10 +38529,10 @@
     </row>
     <row r="26" spans="2:5">
       <c r="B26" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C26" s="90" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="D26" s="90" t="s">
         <v>29</v>
@@ -38528,10 +38543,10 @@
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C27" s="90" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="D27" s="90" t="s">
         <v>30</v>
@@ -38542,10 +38557,10 @@
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C28" s="90" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="D28" s="90" t="s">
         <v>226</v>
@@ -38556,10 +38571,10 @@
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C29" s="90" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="D29" s="90" t="s">
         <v>32</v>
@@ -38570,10 +38585,10 @@
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C30" s="90" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="D30" s="90" t="s">
         <v>33</v>
@@ -38584,10 +38599,10 @@
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="D31" s="90" t="s">
         <v>34</v>
@@ -38598,10 +38613,10 @@
     </row>
     <row r="32" spans="2:5">
       <c r="B32" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C32" s="90" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="D32" s="90" t="s">
         <v>35</v>
@@ -38612,10 +38627,10 @@
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C33" s="90" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D33" s="90" t="s">
         <v>36</v>
@@ -38626,10 +38641,10 @@
     </row>
     <row r="34" spans="2:5">
       <c r="B34" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C34" s="90" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="D34" s="90" t="s">
         <v>37</v>
@@ -38640,10 +38655,10 @@
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="90" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C35" s="90" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D35" s="90" t="s">
         <v>38</v>
@@ -38654,10 +38669,10 @@
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>23</v>
@@ -38668,10 +38683,10 @@
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>24</v>
@@ -38682,10 +38697,10 @@
     </row>
     <row r="38" spans="2:5">
       <c r="B38" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>25</v>
@@ -38696,10 +38711,10 @@
     </row>
     <row r="39" spans="2:5">
       <c r="B39" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>26</v>
@@ -38710,10 +38725,10 @@
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>27</v>
@@ -38724,10 +38739,10 @@
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>28</v>
@@ -38738,10 +38753,10 @@
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>29</v>
@@ -38752,10 +38767,10 @@
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>30</v>
@@ -38766,10 +38781,10 @@
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>226</v>
@@ -38780,10 +38795,10 @@
     </row>
     <row r="45" spans="2:5">
       <c r="B45" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>32</v>
@@ -38794,10 +38809,10 @@
     </row>
     <row r="46" spans="2:5">
       <c r="B46" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>33</v>
@@ -38808,10 +38823,10 @@
     </row>
     <row r="47" spans="2:5">
       <c r="B47" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>34</v>
@@ -38822,10 +38837,10 @@
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>35</v>
@@ -38836,10 +38851,10 @@
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>36</v>
@@ -38850,10 +38865,10 @@
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>37</v>
@@ -38864,10 +38879,10 @@
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="87" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>38</v>
@@ -38878,10 +38893,10 @@
     </row>
     <row r="52" spans="2:5">
       <c r="B52" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="D52" s="91" t="s">
         <v>23</v>
@@ -38892,10 +38907,10 @@
     </row>
     <row r="53" spans="2:5">
       <c r="B53" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="D53" s="91" t="s">
         <v>24</v>
@@ -38906,10 +38921,10 @@
     </row>
     <row r="54" spans="2:5">
       <c r="B54" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="D54" s="91" t="s">
         <v>25</v>
@@ -38920,10 +38935,10 @@
     </row>
     <row r="55" spans="2:5">
       <c r="B55" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="D55" s="91" t="s">
         <v>26</v>
@@ -38934,10 +38949,10 @@
     </row>
     <row r="56" spans="2:5">
       <c r="B56" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="D56" s="91" t="s">
         <v>27</v>
@@ -38948,10 +38963,10 @@
     </row>
     <row r="57" spans="2:5">
       <c r="B57" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D57" s="91" t="s">
         <v>28</v>
@@ -38962,10 +38977,10 @@
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="D58" s="91" t="s">
         <v>29</v>
@@ -38976,10 +38991,10 @@
     </row>
     <row r="59" spans="2:5">
       <c r="B59" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="D59" s="91" t="s">
         <v>30</v>
@@ -38990,10 +39005,10 @@
     </row>
     <row r="60" spans="2:5">
       <c r="B60" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="D60" s="91" t="s">
         <v>226</v>
@@ -39004,10 +39019,10 @@
     </row>
     <row r="61" spans="2:5">
       <c r="B61" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="D61" s="91" t="s">
         <v>32</v>
@@ -39018,10 +39033,10 @@
     </row>
     <row r="62" spans="2:5">
       <c r="B62" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="D62" s="91" t="s">
         <v>33</v>
@@ -39032,10 +39047,10 @@
     </row>
     <row r="63" spans="2:5">
       <c r="B63" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="D63" s="91" t="s">
         <v>34</v>
@@ -39046,10 +39061,10 @@
     </row>
     <row r="64" spans="2:5">
       <c r="B64" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="D64" s="91" t="s">
         <v>35</v>
@@ -39060,10 +39075,10 @@
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="D65" s="91" t="s">
         <v>36</v>
@@ -39074,10 +39089,10 @@
     </row>
     <row r="66" spans="2:5">
       <c r="B66" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="D66" s="91" t="s">
         <v>37</v>
@@ -39088,10 +39103,10 @@
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="87" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D67" s="91" t="s">
         <v>38</v>
@@ -39102,10 +39117,10 @@
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="D68" s="91" t="s">
         <v>23</v>
@@ -39116,10 +39131,10 @@
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D69" s="91" t="s">
         <v>24</v>
@@ -39130,10 +39145,10 @@
     </row>
     <row r="70" spans="2:5">
       <c r="B70" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="D70" s="91" t="s">
         <v>25</v>
@@ -39144,10 +39159,10 @@
     </row>
     <row r="71" spans="2:5">
       <c r="B71" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="D71" s="91" t="s">
         <v>26</v>
@@ -39158,10 +39173,10 @@
     </row>
     <row r="72" spans="2:5">
       <c r="B72" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D72" s="91" t="s">
         <v>27</v>
@@ -39172,10 +39187,10 @@
     </row>
     <row r="73" spans="2:5">
       <c r="B73" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="D73" s="91" t="s">
         <v>28</v>
@@ -39186,10 +39201,10 @@
     </row>
     <row r="74" spans="2:5">
       <c r="B74" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="D74" s="91" t="s">
         <v>29</v>
@@ -39200,10 +39215,10 @@
     </row>
     <row r="75" spans="2:5">
       <c r="B75" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="D75" s="91" t="s">
         <v>30</v>
@@ -39214,10 +39229,10 @@
     </row>
     <row r="76" spans="2:5">
       <c r="B76" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="D76" s="91" t="s">
         <v>226</v>
@@ -39228,10 +39243,10 @@
     </row>
     <row r="77" spans="2:5">
       <c r="B77" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D77" s="91" t="s">
         <v>32</v>
@@ -39242,10 +39257,10 @@
     </row>
     <row r="78" spans="2:5">
       <c r="B78" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="D78" s="91" t="s">
         <v>33</v>
@@ -39256,10 +39271,10 @@
     </row>
     <row r="79" spans="2:5">
       <c r="B79" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="D79" s="91" t="s">
         <v>34</v>
@@ -39270,10 +39285,10 @@
     </row>
     <row r="80" spans="2:5">
       <c r="B80" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="D80" s="91" t="s">
         <v>35</v>
@@ -39284,10 +39299,10 @@
     </row>
     <row r="81" spans="2:5">
       <c r="B81" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D81" s="91" t="s">
         <v>36</v>
@@ -39298,10 +39313,10 @@
     </row>
     <row r="82" spans="2:5">
       <c r="B82" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="D82" s="91" t="s">
         <v>37</v>
@@ -39312,10 +39327,10 @@
     </row>
     <row r="83" spans="2:5">
       <c r="B83" s="87" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="D83" s="91" t="s">
         <v>38</v>
@@ -39528,31 +39543,31 @@
         <v>18</v>
       </c>
       <c r="D11" s="79" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F11" s="79" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G11" s="80" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I11" s="84" t="s">
         <v>23</v>
       </c>
       <c r="J11" s="413" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="K11" s="413" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L11" s="413" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="M11" s="415" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="O11" s="348"/>
     </row>
@@ -39563,31 +39578,31 @@
         <v>16</v>
       </c>
       <c r="D12" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E12" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F12" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G12" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I12" s="41" t="s">
         <v>24</v>
       </c>
       <c r="J12" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K12" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L12" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M12" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N12" s="349"/>
       <c r="O12" s="340"/>
@@ -39599,31 +39614,31 @@
         <v>19</v>
       </c>
       <c r="D13" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E13" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F13" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G13" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I13" s="41" t="s">
         <v>25</v>
       </c>
       <c r="J13" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K13" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L13" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M13" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N13" s="349"/>
       <c r="O13" s="340"/>
@@ -39635,31 +39650,31 @@
         <v>17</v>
       </c>
       <c r="D14" s="71" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="E14" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F14" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G14" s="72" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="I14" s="41" t="s">
         <v>26</v>
       </c>
       <c r="J14" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K14" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L14" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M14" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N14" s="349"/>
       <c r="O14" s="340"/>
@@ -39668,34 +39683,34 @@
       <c r="A15" s="38"/>
       <c r="B15" s="339"/>
       <c r="C15" s="67" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="D15" s="71" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="E15" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F15" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G15" s="72" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="I15" s="41" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K15" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L15" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M15" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N15" s="349"/>
       <c r="O15" s="340"/>
@@ -39704,34 +39719,34 @@
       <c r="A16" s="38"/>
       <c r="B16" s="339"/>
       <c r="C16" s="67" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D16" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E16" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F16" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G16" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I16" s="41" t="s">
         <v>28</v>
       </c>
       <c r="J16" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K16" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L16" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M16" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N16" s="349"/>
       <c r="O16" s="340"/>
@@ -39740,34 +39755,34 @@
       <c r="A17" s="38"/>
       <c r="B17" s="339"/>
       <c r="C17" s="67" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="D17" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E17" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F17" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G17" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I17" s="41" t="s">
         <v>29</v>
       </c>
       <c r="J17" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K17" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L17" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M17" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N17" s="349"/>
       <c r="O17" s="340"/>
@@ -39776,34 +39791,34 @@
       <c r="A18" s="38"/>
       <c r="B18" s="339"/>
       <c r="C18" s="67" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="D18" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E18" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F18" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G18" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I18" s="41" t="s">
         <v>30</v>
       </c>
       <c r="J18" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K18" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L18" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M18" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N18" s="349"/>
       <c r="O18" s="340"/>
@@ -39815,31 +39830,31 @@
         <v>17</v>
       </c>
       <c r="D19" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E19" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F19" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G19" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I19" s="41" t="s">
         <v>226</v>
       </c>
       <c r="J19" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K19" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L19" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M19" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N19" s="349"/>
       <c r="O19" s="340"/>
@@ -39848,34 +39863,34 @@
       <c r="A20" s="38"/>
       <c r="B20" s="339"/>
       <c r="C20" s="40" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="D20" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E20" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F20" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G20" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I20" s="41" t="s">
         <v>32</v>
       </c>
       <c r="J20" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K20" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L20" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M20" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N20" s="349"/>
       <c r="O20" s="340"/>
@@ -39884,34 +39899,34 @@
       <c r="A21" s="38"/>
       <c r="B21" s="339"/>
       <c r="C21" s="39" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="D21" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E21" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F21" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G21" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I21" s="41" t="s">
         <v>33</v>
       </c>
       <c r="J21" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K21" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L21" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M21" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N21" s="349"/>
       <c r="O21" s="340"/>
@@ -39920,34 +39935,34 @@
       <c r="A22" s="38"/>
       <c r="B22" s="339"/>
       <c r="C22" s="39" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="D22" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E22" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F22" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G22" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I22" s="41" t="s">
         <v>34</v>
       </c>
       <c r="J22" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K22" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L22" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M22" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N22" s="349"/>
       <c r="O22" s="340"/>
@@ -39956,34 +39971,34 @@
       <c r="A23" s="38"/>
       <c r="B23" s="339"/>
       <c r="C23" s="40" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="D23" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E23" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F23" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G23" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I23" s="41" t="s">
         <v>35</v>
       </c>
       <c r="J23" s="414" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="K23" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L23" s="414" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="M23" s="416" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="N23" s="349"/>
       <c r="O23" s="340"/>
@@ -39995,31 +40010,31 @@
         <v>20</v>
       </c>
       <c r="D24" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="E24" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F24" s="71" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="G24" s="72" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="I24" s="41" t="s">
         <v>36</v>
       </c>
       <c r="J24" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K24" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L24" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M24" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N24" s="349"/>
       <c r="O24" s="340"/>
@@ -40036,16 +40051,16 @@
         <v>37</v>
       </c>
       <c r="J25" s="414" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="K25" s="414" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L25" s="414" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M25" s="416" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="N25" s="349"/>
       <c r="O25" s="340"/>
@@ -40062,16 +40077,16 @@
         <v>38</v>
       </c>
       <c r="J26" s="417" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="K26" s="417" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L26" s="417" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="M26" s="418" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="N26" s="349"/>
       <c r="O26" s="340"/>
@@ -40279,7 +40294,7 @@
       <c r="E2" s="104"/>
       <c r="G2" s="106"/>
       <c r="H2" s="98" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="I2" s="523" t="s">
         <v>123</v>
@@ -40296,7 +40311,7 @@
     <row r="3" spans="1:17" s="69" customFormat="1" ht="22.5" customHeight="1">
       <c r="A3" s="101"/>
       <c r="B3" s="69" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="D3" s="107"/>
       <c r="E3" s="100"/>
@@ -40670,7 +40685,7 @@
         <v>115</v>
       </c>
       <c r="E16" s="520" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="F16" s="521"/>
       <c r="G16" s="521"/>
@@ -40693,7 +40708,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="520" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="F17" s="521"/>
       <c r="G17" s="521"/>
@@ -40717,7 +40732,7 @@
         <v>117</v>
       </c>
       <c r="E18" s="520" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="F18" s="521"/>
       <c r="G18" s="521"/>
@@ -40738,7 +40753,7 @@
         <v>118</v>
       </c>
       <c r="E19" s="520" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="F19" s="521"/>
       <c r="G19" s="521"/>
@@ -40759,7 +40774,7 @@
         <v>119</v>
       </c>
       <c r="E20" s="520" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="F20" s="521"/>
       <c r="G20" s="521"/>
@@ -40779,7 +40794,7 @@
         <v>120</v>
       </c>
       <c r="E21" s="520" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="F21" s="521"/>
       <c r="G21" s="521"/>
@@ -40797,10 +40812,10 @@
       <c r="B22" s="125"/>
       <c r="C22" s="103"/>
       <c r="D22" s="410" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="E22" s="520" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="F22" s="521"/>
       <c r="G22" s="521"/>

</xml_diff>